<commit_message>
Updated PBL excel documentation + added newly added columns to Building excel
</commit_message>
<xml_diff>
--- a/data_ProjectTemplate/Buildings_ProjectTemplate.xlsx
+++ b/data_ProjectTemplate/Buildings_ProjectTemplate.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AteHe\Desktop\Modellen\LUX_ProjectTemplate\data_ProjectTemplate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Bas\Desktop\Github\data_Generic\data_ProjectTemplate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13149339-643D-44BF-BF53-D5A0B0256AF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C70D194F-3977-4A92-BCAE-FBD97E9F9D11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{99A50208-934F-4EDD-BF51-6D238E9C57FC}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{99A50208-934F-4EDD-BF51-6D238E9C57FC}"/>
   </bookViews>
   <sheets>
     <sheet name="buildings" sheetId="4" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">buildings!$A$1:$X$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">buildings!$A$1:$AI$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,9 +43,10 @@
   <authors>
     <author>Ate Hempenius</author>
     <author>Luc Sol</author>
+    <author>Bas Dekker</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{4FF04E4C-5292-4BEB-9F6E-79CE20556081}">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{4C13E7C5-8699-4852-866B-172874E240FD}">
       <text>
         <r>
           <rPr>
@@ -70,7 +71,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{57152F91-9E06-4D31-9EEF-EA9B213461F2}">
+    <comment ref="B1" authorId="0" shapeId="0" xr:uid="{16F1B0E8-7C62-4D5A-B778-A1FCAEE03988}">
       <text>
         <r>
           <rPr>
@@ -95,7 +96,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{63B43FE4-2DFE-458F-AA88-0AD3D1781F0B}">
+    <comment ref="C1" authorId="1" shapeId="0" xr:uid="{6B59763B-138A-49E4-B992-46EB31FE2842}">
       <text>
         <r>
           <rPr>
@@ -121,7 +122,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{3D1D533C-5B41-43B7-9FCE-CE4797AADFC4}">
+    <comment ref="D1" authorId="1" shapeId="0" xr:uid="{BB269F86-FB67-4A8F-83EF-1DF2C1A35790}">
       <text>
         <r>
           <rPr>
@@ -148,7 +149,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{9DB1F80B-7770-448F-B7C5-B95C6227531F}">
+    <comment ref="E1" authorId="1" shapeId="0" xr:uid="{FB4D2EDD-CBDE-4AC2-BD00-1EDA4BE11CEE}">
       <text>
         <r>
           <rPr>
@@ -174,7 +175,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{22E69195-E33A-46EC-B4A6-7699828DF447}">
+    <comment ref="F1" authorId="1" shapeId="0" xr:uid="{B9FD15B5-646C-4F09-BC9E-D3B249DC462C}">
       <text>
         <r>
           <rPr>
@@ -200,7 +201,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{F1CF16E5-D70A-40ED-8B78-A5BC817F8BCC}">
+    <comment ref="G1" authorId="1" shapeId="0" xr:uid="{650D67DA-5976-46B1-B2B2-8FA6B77E34D4}">
       <text>
         <r>
           <rPr>
@@ -226,7 +227,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H1" authorId="1" shapeId="0" xr:uid="{1EAEF5C4-DB6F-463A-9305-C54F332EB207}">
+    <comment ref="H1" authorId="1" shapeId="0" xr:uid="{58F6014B-EAEA-43E1-97B8-5FB1E87F14AD}">
       <text>
         <r>
           <rPr>
@@ -253,7 +254,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{5A795051-8748-4EEF-851C-A7F6C88CA63B}">
+    <comment ref="I1" authorId="1" shapeId="0" xr:uid="{634346CB-5BD7-464D-9991-CAD5C1E51C7D}">
       <text>
         <r>
           <rPr>
@@ -279,7 +280,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{0180DFDE-884B-49DC-AAAB-8EF8231D6AF7}">
+    <comment ref="J1" authorId="1" shapeId="0" xr:uid="{27E12FF1-A5FB-4BBC-9643-91F905BE13B7}">
       <text>
         <r>
           <rPr>
@@ -304,7 +305,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{DEB1C7F1-4305-4F7A-A3C4-2A9AFFA49F4B}">
+    <comment ref="K1" authorId="1" shapeId="0" xr:uid="{697A9B81-D74E-4603-83D8-62B712560483}">
       <text>
         <r>
           <rPr>
@@ -329,7 +330,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L1" authorId="1" shapeId="0" xr:uid="{67A75FA9-0BD1-4CD7-B438-8099B3F91CFD}">
+    <comment ref="L1" authorId="1" shapeId="0" xr:uid="{7E67C321-ACE5-4A3F-8791-8CB5A66B7772}">
       <text>
         <r>
           <rPr>
@@ -358,7 +359,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{A69ACB59-63D9-405D-B1E7-8C5FCD486732}">
+    <comment ref="M1" authorId="1" shapeId="0" xr:uid="{566B1C09-CD85-4A88-AAAB-71AFF4A3E66C}">
       <text>
         <r>
           <rPr>
@@ -383,7 +384,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N1" authorId="1" shapeId="0" xr:uid="{524DA785-47C5-4088-BB61-39BB2001FD08}">
+    <comment ref="N1" authorId="1" shapeId="0" xr:uid="{717C5184-6966-4283-B2F0-AA6EAFC7318D}">
       <text>
         <r>
           <rPr>
@@ -411,7 +412,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O1" authorId="1" shapeId="0" xr:uid="{C8777648-5A5B-4EBB-828A-593EF2D45AFE}">
+    <comment ref="O1" authorId="1" shapeId="0" xr:uid="{7DDB3FEC-04D3-4259-B18F-2D8EF995AF82}">
       <text>
         <r>
           <rPr>
@@ -437,7 +438,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P1" authorId="1" shapeId="0" xr:uid="{819AAD6C-12F9-4998-BED6-422C1A07BFFC}">
+    <comment ref="P1" authorId="1" shapeId="0" xr:uid="{9619647D-DD6B-445C-834F-98143E859C8C}">
       <text>
         <r>
           <rPr>
@@ -463,7 +464,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q1" authorId="1" shapeId="0" xr:uid="{C1656C3D-075F-46BD-BC2F-A2B624759EAD}">
+    <comment ref="Q1" authorId="1" shapeId="0" xr:uid="{66C1476F-070C-400B-B611-AE96B262EA65}">
       <text>
         <r>
           <rPr>
@@ -488,7 +489,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R1" authorId="1" shapeId="0" xr:uid="{313BE7C2-A32D-4855-9081-1060871BCACE}">
+    <comment ref="R1" authorId="1" shapeId="0" xr:uid="{1F8EE453-6B20-438F-8097-F3BFF165B50E}">
       <text>
         <r>
           <rPr>
@@ -513,7 +514,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{FA84333F-E852-4BA6-ADC3-4C18ED3E848F}">
+    <comment ref="S1" authorId="1" shapeId="0" xr:uid="{425BBA42-7F3A-413D-8BF2-F6914BEB9F7C}">
       <text>
         <r>
           <rPr>
@@ -538,7 +539,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T1" authorId="1" shapeId="0" xr:uid="{AD24B6AB-1158-43E8-842F-4D714C92F510}">
+    <comment ref="T1" authorId="1" shapeId="0" xr:uid="{5FCC0FA5-AEC9-4216-9A4F-33C6B7CEAEE5}">
       <text>
         <r>
           <rPr>
@@ -564,7 +565,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="U1" authorId="1" shapeId="0" xr:uid="{6FABADF5-9806-436F-81EC-5A02247424E9}">
+    <comment ref="U1" authorId="1" shapeId="0" xr:uid="{2157A997-7256-480A-B18F-60B7C33EE6D2}">
       <text>
         <r>
           <rPr>
@@ -590,7 +591,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="V1" authorId="1" shapeId="0" xr:uid="{D6946C39-BC7B-45E2-98F8-4E43651FB286}">
+    <comment ref="V1" authorId="1" shapeId="0" xr:uid="{6750B72F-E6F8-4AA7-B91E-A948E4ACE7AD}">
       <text>
         <r>
           <rPr>
@@ -615,7 +616,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W1" authorId="1" shapeId="0" xr:uid="{EC4AD394-CB46-40F7-891D-56876710C581}">
+    <comment ref="W1" authorId="1" shapeId="0" xr:uid="{DB513A7B-022D-4B6A-99BB-0AA9A1939F38}">
       <text>
         <r>
           <rPr>
@@ -639,7 +640,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="1" shapeId="0" xr:uid="{F61542DC-50BE-45B0-BDA5-41015EE1B282}">
+    <comment ref="X1" authorId="1" shapeId="0" xr:uid="{39B0F5CD-E78A-4E34-8EA8-B4F7D8813A1A}">
       <text>
         <r>
           <rPr>
@@ -662,6 +663,375 @@
 String (mandatory)
 Polygon or MultiPolygon from QGIS
 </t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="2" shapeId="0" xr:uid="{7E13EC75-793A-40EB-8D8D-3D6843B8B466}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">Bas Dekker:
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>double</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve"> </t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>[Optional]
+Contains the currently installed PV kWp for the address</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Z1" authorId="2" shapeId="0" xr:uid="{3F48ED9A-6710-4EE7-8EA1-9D8E22461B49}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+double [Optional] 
+Contains the maximum potential for installed PV kWp for the address</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AA1" authorId="2" shapeId="0" xr:uid="{CA1C2A37-461F-47A2-96EA-78E9DE2DA2B4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+boolean [optional]
+Has private parking spot at address (TRUE if does not FALSE)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AB1" authorId="2" shapeId="0" xr:uid="{6B5673B2-2E2D-40AB-A8B8-1B074515A644}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Description of dwelling type</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AC1" authorId="2" shapeId="0" xr:uid="{A745210B-D882-4EDE-BB1A-823F9ADB1502}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+SBI code</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD1" authorId="2" shapeId="0" xr:uid="{1DD00F5A-ED4C-482B-91E5-9149AF10B238}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Additional description to the dwelling type
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AE1" authorId="2" shapeId="0" xr:uid="{B7620385-ACC2-4726-965C-0EB89E6DBA6A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Type of cooking installation: gasfornuis/inductie
+Not implemented yet</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF1" authorId="2" shapeId="0" xr:uid="{6380C347-3206-49F6-925A-F3C7E08F1B5C}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+Installed type of heating for address
+Not implemented yet</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG1" authorId="2" shapeId="0" xr:uid="{D82C59A4-E903-4F1A-9AE2-680F973F3871}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Integer [optional]
+PBL-based
+PBL Dwellingtypes:
+1: vrijstaand
+2: 2-onder-1 kap
+3: rijwoning hoekwoning
+4: rijwoning tussenwoning
+5: appartementen t/m 4 (meergezinswoningen t/m 4 verdiepingen)
+6: appartementen 5&gt;= (meergezinswoningen 5 of meer verdiepingen)</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AH1" authorId="2" shapeId="0" xr:uid="{098504A7-C35B-4755-AE93-35BCFB975ACE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Integer [optional]
+PBL-based
+OwnershipType:
+0: Koop
+1: Particulier Huur
+2: Sociale Huur</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AI1" authorId="2" shapeId="0" xr:uid="{0AEF554D-3521-459D-AE9D-09BD6E1322F3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+String [optional]
+PBL-based
+(Insulation label):
+A+
+A
+B
+C
+D
+E
+F
+G</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AJ1" authorId="2" shapeId="0" xr:uid="{65515451-44AD-4EAA-B21D-CDDDC4E0BF0F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+double [optional]
+PBL-based
+Regional climate correction factor: used to compensate for regional climate differences between models for heating consumption</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AK1" authorId="2" shapeId="0" xr:uid="{CCB74FF6-9A18-47F6-89E9-5D2B4AEE4A96}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Bas Dekker:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+double [optional]
+PBL-based
+local factor: factor to compensate for local differences between neighbourhoods that affect heating consumption</t>
         </r>
       </text>
     </comment>
@@ -670,7 +1040,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>polygon</t>
   </si>
@@ -742,13 +1112,52 @@
   </si>
   <si>
     <t>gas_consumption_m3pa</t>
+  </si>
+  <si>
+    <t>pv_installed_kwp</t>
+  </si>
+  <si>
+    <t>pv_potential_kwp</t>
+  </si>
+  <si>
+    <t>private_parking</t>
+  </si>
+  <si>
+    <t>house_type</t>
+  </si>
+  <si>
+    <t>sbi_code</t>
+  </si>
+  <si>
+    <t>building_subtype</t>
+  </si>
+  <si>
+    <t>dwelling_type</t>
+  </si>
+  <si>
+    <t>ownership_type</t>
+  </si>
+  <si>
+    <t>insulation_label</t>
+  </si>
+  <si>
+    <t>regional_climate_correction_factor</t>
+  </si>
+  <si>
+    <t>local_factor</t>
+  </si>
+  <si>
+    <t>cooking_type</t>
+  </si>
+  <si>
+    <t>heating_type</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -768,6 +1177,19 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1145,34 +1567,48 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFCD9D70-6DEB-4390-947E-55D38CEBDCD5}">
-  <dimension ref="A1:X1"/>
-  <sheetFormatPr defaultColWidth="10.1796875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AK1"/>
+  <sheetFormatPr defaultColWidth="10.21875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.81640625" customWidth="1"/>
-    <col min="2" max="2" width="41.54296875" customWidth="1"/>
-    <col min="3" max="3" width="15.7265625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="7.6328125" customWidth="1"/>
-    <col min="9" max="9" width="9.81640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="7.81640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="26.54296875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="5.26953125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="41.08984375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="91.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="21.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="28.54296875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="22.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="7.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="23" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="3.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="28.44140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="15" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="31.33203125" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="11.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
@@ -1245,9 +1681,47 @@
       <c r="X1" s="1" t="s">
         <v>0</v>
       </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="AB1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>34</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:X1" xr:uid="{CFCD9D70-6DEB-4390-947E-55D38CEBDCD5}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>

</xml_diff>